<commit_message>
fix(scripts): parser ignora linhas de totalizador numerico
</commit_message>
<xml_diff>
--- a/scripts/tests/fixtures/mini-matriculados.xlsx
+++ b/scripts/tests/fixtures/mini-matriculados.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="12">
   <si>
     <t>MATERNAL - MATUTINO</t>
   </si>
@@ -33,6 +33,15 @@
   </si>
   <si>
     <t>Manuela Margarida Barros</t>
+  </si>
+  <si>
+    <t>INFANTIL 5 - MATUTINO</t>
+  </si>
+  <si>
+    <t>Pedro Silva</t>
+  </si>
+  <si>
+    <t>Maria Souza</t>
   </si>
   <si>
     <t>3º ANO - B</t>
@@ -415,7 +424,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A3:E10"/>
+  <dimension ref="A3:E17"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
@@ -475,6 +484,46 @@
       </c>
       <c r="E10">
         <v>800</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D12" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D13" t="s">
+        <v>1</v>
+      </c>
+      <c r="E13" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="C14">
+        <v>1</v>
+      </c>
+      <c r="D14" t="s">
+        <v>8</v>
+      </c>
+      <c r="E14">
+        <v>700</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="C15">
+        <v>2</v>
+      </c>
+      <c r="D15" t="s">
+        <v>9</v>
+      </c>
+      <c r="E15">
+        <v>720</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D17">
+        <v>1420</v>
       </c>
     </row>
   </sheetData>
@@ -490,7 +539,7 @@
   <sheetData>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D2" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
@@ -506,7 +555,7 @@
         <v>1</v>
       </c>
       <c r="D4" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="E4">
         <v>700</v>

</xml_diff>